<commit_message>
Veri güncellendi: 2026-04-24 05:58
</commit_message>
<xml_diff>
--- a/BISTTemelVeriler.xlsx
+++ b/BISTTemelVeriler.xlsx
@@ -1432,10 +1432,10 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>3.6</v>
+        <v>3.3</v>
       </c>
       <c r="E10" t="n">
-        <v>1.4</v>
+        <v>1.3</v>
       </c>
       <c r="P10" t="n">
         <v>203.3863</v>
@@ -1505,13 +1505,10 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>8.300000000000001</v>
-      </c>
-      <c r="E11" t="n">
+        <v>12</v>
+      </c>
+      <c r="O11" t="n">
         <v>0.8</v>
-      </c>
-      <c r="O11" t="n">
-        <v>0.4</v>
       </c>
       <c r="P11" t="n">
         <v>26.96</v>
@@ -2074,19 +2071,19 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>12.5</v>
+        <v>18.7</v>
       </c>
       <c r="D17" t="n">
-        <v>6.9</v>
+        <v>8</v>
       </c>
       <c r="E17" t="n">
-        <v>1.1</v>
+        <v>1.2</v>
       </c>
       <c r="F17" t="n">
-        <v>1.2</v>
+        <v>1.3</v>
       </c>
       <c r="O17" t="n">
-        <v>1.2</v>
+        <v>1.3</v>
       </c>
       <c r="P17" t="n">
         <v>167.4</v>
@@ -2559,13 +2556,13 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>3</v>
+        <v>1.9</v>
       </c>
       <c r="E22" t="n">
-        <v>0.8</v>
+        <v>0.5</v>
       </c>
       <c r="O22" t="n">
-        <v>37.2</v>
+        <v>36.7</v>
       </c>
       <c r="P22" t="n">
         <v>7</v>
@@ -4626,10 +4623,10 @@
         </is>
       </c>
       <c r="C44" t="n">
-        <v>4.5</v>
+        <v>3.2</v>
       </c>
       <c r="E44" t="n">
-        <v>2</v>
+        <v>1.4</v>
       </c>
       <c r="P44" t="n">
         <v>101.7159</v>
@@ -4702,10 +4699,10 @@
         <v>2.6</v>
       </c>
       <c r="E45" t="n">
-        <v>0.8</v>
+        <v>0.7</v>
       </c>
       <c r="O45" t="n">
-        <v>39.4</v>
+        <v>36.3</v>
       </c>
       <c r="P45" t="n">
         <v>23.9669</v>
@@ -4883,14 +4880,17 @@
           <t>Arçelik Hisse Senedi</t>
         </is>
       </c>
+      <c r="C47" t="n">
+        <v>13.4</v>
+      </c>
       <c r="D47" t="n">
-        <v>4.2</v>
+        <v>5.1</v>
       </c>
       <c r="E47" t="n">
-        <v>0.9</v>
+        <v>1</v>
       </c>
       <c r="F47" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="O47" t="n">
         <v>0.4</v>
@@ -4920,13 +4920,13 @@
         </is>
       </c>
       <c r="V47" t="n">
-        <v>70390.60000000001</v>
+        <v>73314.5</v>
       </c>
       <c r="W47" t="n">
         <v>675.7</v>
       </c>
       <c r="X47" t="n">
-        <v>-8355.700000000001</v>
+        <v>-1816.8</v>
       </c>
       <c r="Y47" t="inlineStr">
         <is>
@@ -7703,17 +7703,8 @@
           <t>Aygaz Hisse Senedi</t>
         </is>
       </c>
-      <c r="C75" t="n">
-        <v>6.9</v>
-      </c>
-      <c r="D75" t="n">
-        <v>16.9</v>
-      </c>
-      <c r="E75" t="n">
-        <v>0.7</v>
-      </c>
       <c r="F75" t="n">
-        <v>0.5</v>
+        <v>35.9</v>
       </c>
       <c r="O75" t="n">
         <v>0.5</v>
@@ -9943,16 +9934,16 @@
         </is>
       </c>
       <c r="C97" t="n">
-        <v>14.6</v>
+        <v>16</v>
       </c>
       <c r="D97" t="n">
         <v>6.5</v>
       </c>
       <c r="E97" t="n">
-        <v>1.6</v>
+        <v>1.7</v>
       </c>
       <c r="F97" t="n">
-        <v>0.5</v>
+        <v>0.4</v>
       </c>
       <c r="O97" t="n">
         <v>0.5</v>
@@ -13427,16 +13418,16 @@
         </is>
       </c>
       <c r="C131" t="n">
-        <v>11</v>
+        <v>10.4</v>
       </c>
       <c r="D131" t="n">
-        <v>5.5</v>
+        <v>5.4</v>
       </c>
       <c r="E131" t="n">
-        <v>2.3</v>
+        <v>2.2</v>
       </c>
       <c r="F131" t="n">
-        <v>1</v>
+        <v>0.9</v>
       </c>
       <c r="O131" t="n">
         <v>1</v>
@@ -14139,19 +14130,19 @@
         </is>
       </c>
       <c r="C138" t="n">
-        <v>8</v>
+        <v>12.3</v>
       </c>
       <c r="D138" t="n">
-        <v>6</v>
+        <v>6.9</v>
       </c>
       <c r="E138" t="n">
-        <v>1.8</v>
+        <v>1.7</v>
       </c>
       <c r="F138" t="n">
-        <v>1.3</v>
+        <v>1.4</v>
       </c>
       <c r="O138" t="n">
-        <v>1.3</v>
+        <v>1.4</v>
       </c>
       <c r="P138" t="n">
         <v>46.4037</v>
@@ -15220,13 +15211,13 @@
         </is>
       </c>
       <c r="V148" t="n">
-        <v>13949.8</v>
+        <v>16106.3</v>
       </c>
       <c r="W148" t="n">
         <v>1078.3</v>
       </c>
       <c r="X148" t="n">
-        <v>2215.1</v>
+        <v>737.7</v>
       </c>
       <c r="Y148" t="inlineStr">
         <is>
@@ -17151,7 +17142,7 @@
         </is>
       </c>
       <c r="C168" t="n">
-        <v>7.2</v>
+        <v>7.6</v>
       </c>
       <c r="D168" t="n">
         <v>3.6</v>
@@ -20911,19 +20902,19 @@
         </is>
       </c>
       <c r="C205" t="n">
-        <v>10.2</v>
+        <v>8</v>
       </c>
       <c r="D205" t="n">
-        <v>6.4</v>
+        <v>5</v>
       </c>
       <c r="E205" t="n">
-        <v>1.1</v>
+        <v>0.9</v>
       </c>
       <c r="F205" t="n">
+        <v>1</v>
+      </c>
+      <c r="O205" t="n">
         <v>1.4</v>
-      </c>
-      <c r="O205" t="n">
-        <v>2</v>
       </c>
       <c r="P205" t="n">
         <v>82.1562</v>
@@ -23779,10 +23770,10 @@
         </is>
       </c>
       <c r="C233" t="n">
-        <v>8.800000000000001</v>
+        <v>9.5</v>
       </c>
       <c r="D233" t="n">
-        <v>5.9</v>
+        <v>6.3</v>
       </c>
       <c r="E233" t="n">
         <v>1.9</v>
@@ -35184,19 +35175,19 @@
         </is>
       </c>
       <c r="C346" t="n">
-        <v>10.3</v>
+        <v>12.1</v>
       </c>
       <c r="D346" t="n">
-        <v>2</v>
+        <v>2.1</v>
       </c>
       <c r="E346" t="n">
-        <v>1.3</v>
+        <v>1.5</v>
       </c>
       <c r="F346" t="n">
-        <v>0.5</v>
+        <v>0.4</v>
       </c>
       <c r="O346" t="n">
-        <v>0.5</v>
+        <v>0.4</v>
       </c>
       <c r="P346" t="n">
         <v>14.14</v>
@@ -37209,16 +37200,16 @@
         </is>
       </c>
       <c r="C366" t="n">
-        <v>10.9</v>
+        <v>10.4</v>
       </c>
       <c r="D366" t="n">
-        <v>5</v>
+        <v>4.7</v>
       </c>
       <c r="E366" t="n">
         <v>1.4</v>
       </c>
       <c r="F366" t="n">
-        <v>1.1</v>
+        <v>1</v>
       </c>
       <c r="O366" t="n">
         <v>1.1</v>
@@ -37621,19 +37612,19 @@
         </is>
       </c>
       <c r="C370" t="n">
-        <v>4.1</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="D370" t="n">
-        <v>4.3</v>
+        <v>3.8</v>
       </c>
       <c r="E370" t="n">
-        <v>1.7</v>
+        <v>2.1</v>
       </c>
       <c r="F370" t="n">
-        <v>1.4</v>
+        <v>1.2</v>
       </c>
       <c r="O370" t="n">
-        <v>1.5</v>
+        <v>1.3</v>
       </c>
       <c r="P370" t="n">
         <v>131.8</v>
@@ -39156,13 +39147,13 @@
         </is>
       </c>
       <c r="C386" t="n">
-        <v>6.3</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="D386" t="n">
-        <v>2.4</v>
+        <v>2.7</v>
       </c>
       <c r="E386" t="n">
-        <v>1.8</v>
+        <v>1.9</v>
       </c>
       <c r="F386" t="n">
         <v>0.5</v>
@@ -40397,13 +40388,13 @@
         </is>
       </c>
       <c r="C398" t="n">
-        <v>7.8</v>
+        <v>3.1</v>
       </c>
       <c r="D398" t="n">
         <v>2.5</v>
       </c>
       <c r="E398" t="n">
-        <v>0.9</v>
+        <v>0.8</v>
       </c>
       <c r="F398" t="n">
         <v>0.2</v>
@@ -41296,16 +41287,19 @@
         </is>
       </c>
       <c r="C407" t="n">
-        <v>12.6</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="D407" t="n">
-        <v>5</v>
+        <v>4.2</v>
+      </c>
+      <c r="E407" t="n">
+        <v>5.5</v>
       </c>
       <c r="F407" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="O407" t="n">
         <v>1.3</v>
-      </c>
-      <c r="O407" t="n">
-        <v>1.4</v>
       </c>
       <c r="P407" t="n">
         <v>408</v>
@@ -44297,13 +44291,13 @@
         </is>
       </c>
       <c r="C436" t="n">
-        <v>11.9</v>
+        <v>12.3</v>
       </c>
       <c r="D436" t="n">
         <v>5.9</v>
       </c>
       <c r="E436" t="n">
-        <v>1.5</v>
+        <v>1.6</v>
       </c>
       <c r="F436" t="n">
         <v>1.6</v>
@@ -46452,17 +46446,8 @@
           <t>Petkim Hisse Senedi</t>
         </is>
       </c>
-      <c r="D457" t="n">
-        <v>18.2</v>
-      </c>
-      <c r="E457" t="n">
-        <v>1.3</v>
-      </c>
-      <c r="F457" t="n">
+      <c r="O457" t="n">
         <v>0.8</v>
-      </c>
-      <c r="O457" t="n">
-        <v>0.9</v>
       </c>
       <c r="P457" t="n">
         <v>17.29</v>
@@ -46644,7 +46629,7 @@
         </is>
       </c>
       <c r="C459" t="n">
-        <v>5.6</v>
+        <v>5.5</v>
       </c>
       <c r="D459" t="n">
         <v>3.9</v>
@@ -52870,13 +52855,13 @@
         </is>
       </c>
       <c r="C520" t="n">
-        <v>17.6</v>
+        <v>3.9</v>
       </c>
       <c r="D520" t="n">
-        <v>2.4</v>
+        <v>1.4</v>
       </c>
       <c r="E520" t="n">
-        <v>0.6</v>
+        <v>0.5</v>
       </c>
       <c r="F520" t="n">
         <v>0.1</v>
@@ -54082,19 +54067,19 @@
         </is>
       </c>
       <c r="C532" t="n">
-        <v>12.1</v>
+        <v>18.2</v>
       </c>
       <c r="D532" t="n">
-        <v>4.2</v>
+        <v>4.6</v>
       </c>
       <c r="E532" t="n">
-        <v>0.9</v>
+        <v>1</v>
       </c>
       <c r="F532" t="n">
-        <v>1.3</v>
+        <v>1.4</v>
       </c>
       <c r="O532" t="n">
-        <v>1.6</v>
+        <v>1.8</v>
       </c>
       <c r="P532" t="n">
         <v>286</v>
@@ -54276,10 +54261,13 @@
         </is>
       </c>
       <c r="C534" t="n">
-        <v>6.8</v>
+        <v>7.8</v>
       </c>
       <c r="D534" t="n">
         <v>2.1</v>
+      </c>
+      <c r="E534" t="n">
+        <v>1</v>
       </c>
       <c r="F534" t="n">
         <v>0.9</v>
@@ -55097,19 +55085,19 @@
         </is>
       </c>
       <c r="C542" t="n">
-        <v>4</v>
+        <v>2.6</v>
       </c>
       <c r="D542" t="n">
-        <v>4.1</v>
+        <v>3.1</v>
       </c>
       <c r="E542" t="n">
-        <v>0.3</v>
+        <v>0.2</v>
       </c>
       <c r="F542" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="O542" t="n">
         <v>0.6</v>
-      </c>
-      <c r="O542" t="n">
-        <v>0.8</v>
       </c>
       <c r="P542" t="n">
         <v>276.75</v>
@@ -55769,13 +55757,13 @@
         </is>
       </c>
       <c r="C549" t="n">
-        <v>3.6</v>
+        <v>4.4</v>
       </c>
       <c r="D549" t="n">
-        <v>3.7</v>
+        <v>4.6</v>
       </c>
       <c r="E549" t="n">
-        <v>1.3</v>
+        <v>1.4</v>
       </c>
       <c r="F549" t="n">
         <v>0.3</v>
@@ -56824,19 +56812,19 @@
         </is>
       </c>
       <c r="C560" t="n">
-        <v>3.3</v>
+        <v>2.8</v>
       </c>
       <c r="D560" t="n">
         <v>1.9</v>
       </c>
       <c r="E560" t="n">
-        <v>0.8</v>
+        <v>0.7</v>
       </c>
       <c r="F560" t="n">
         <v>0.8</v>
       </c>
       <c r="O560" t="n">
-        <v>0.9</v>
+        <v>0.8</v>
       </c>
       <c r="P560" t="n">
         <v>57.2</v>
@@ -56909,13 +56897,13 @@
         </is>
       </c>
       <c r="C561" t="n">
-        <v>8</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="D561" t="n">
-        <v>4.8</v>
+        <v>5</v>
       </c>
       <c r="E561" t="n">
-        <v>2.2</v>
+        <v>2.1</v>
       </c>
       <c r="F561" t="n">
         <v>0.6</v>
@@ -57509,7 +57497,7 @@
         <v>4.2</v>
       </c>
       <c r="E567" t="n">
-        <v>1.8</v>
+        <v>1.5</v>
       </c>
       <c r="P567" t="n">
         <v>11.51</v>
@@ -57885,10 +57873,10 @@
         </is>
       </c>
       <c r="C571" t="n">
-        <v>3.4</v>
+        <v>4.2</v>
       </c>
       <c r="D571" t="n">
-        <v>3</v>
+        <v>3.2</v>
       </c>
       <c r="E571" t="n">
         <v>0.9</v>
@@ -58221,13 +58209,13 @@
         </is>
       </c>
       <c r="V574" t="n">
-        <v>12913.5</v>
+        <v>13712</v>
       </c>
       <c r="W574" t="n">
         <v>750</v>
       </c>
       <c r="X574" t="n">
-        <v>-287.2</v>
+        <v>-130.9</v>
       </c>
       <c r="Y574" t="inlineStr">
         <is>

</xml_diff>